<commit_message>
EGO Master LIVE: Dealers, Architects and People
</commit_message>
<xml_diff>
--- a/ego/Big-E-Upload-Template.xlsx
+++ b/ego/Big-E-Upload-Template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="How to fill" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Architect firms" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Architect people" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Clients" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="People (no company)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Products &amp; warehouses" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Lists" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
@@ -547,7 +547,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Companies first, then the people who work in them, then the clients. A person's company is written exactly as its name on the companies sheet.</t>
+          <t>Companies first, then the people who work in them, then people with no company. A person's company is written exactly as its name on the companies sheet.</t>
         </is>
       </c>
     </row>
@@ -690,12 +690,12 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Clients</t>
+          <t>People (no company)</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Clients who are not under any dealer or architect: an individual, or a firm on its own (builder, hotel, corporate). One row each.</t>
+          <t>People with no company: an individual, or a firm on its own (builder, hotel, corporate). Not a dealer's or an architect's staff: they go on the people sheets. One row each.</t>
         </is>
       </c>
     </row>
@@ -5395,7 +5395,7 @@
   <dimension ref="A1:S201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
     <col width="29" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
@@ -5419,7 +5419,7 @@
     <row r="1" ht="48" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Client name (person or firm) *</t>
+          <t>Person or firm name *</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">

</xml_diff>

<commit_message>
EGO Master LIVE: editable lists
</commit_message>
<xml_diff>
--- a/ego/Big-E-Upload-Template.xlsx
+++ b/ego/Big-E-Upload-Template.xlsx
@@ -6967,31 +6967,31 @@
   </sheetData>
   <dataValidations count="9">
     <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$A$1:$A$2</formula1>
+      <formula1>=Lists!$A$2:$A$3</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$B$1:$B$16</formula1>
+      <formula1>=Lists!$B$2:$B$17</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$C$1:$C$22</formula1>
+      <formula1>=Lists!$C$2:$C$23</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." promptTitle="Pick or type" prompt="Pick from the list, or type several separated by commas." type="list">
-      <formula1>=Lists!$D$1:$D$22</formula1>
+      <formula1>=Lists!$D$2:$D$23</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." promptTitle="Pick or type" prompt="Pick from the list, or type it." type="list">
-      <formula1>=Lists!$E$1:$E$2</formula1>
+      <formula1>=Lists!$E$2:$E$3</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$F$1:$F$3</formula1>
+      <formula1>=Lists!$F$2:$F$4</formula1>
     </dataValidation>
     <dataValidation sqref="R2:R1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$G$1:$G$13</formula1>
+      <formula1>=Lists!$G$2:$G$14</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$H$1:$H$3</formula1>
+      <formula1>=Lists!$H$2:$H$4</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$I$1:$I$2</formula1>
+      <formula1>=Lists!$I$2:$I$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12383,10 +12383,10 @@
       <formula1>='Architect firms'!$B$3:$B$1000</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$J$1:$J$16</formula1>
+      <formula1>=Lists!$J$2:$J$17</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$K$1:$K$2</formula1>
+      <formula1>=Lists!$K$2:$K$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18039,19 +18039,19 @@
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$L$1:$L$9</formula1>
+      <formula1>=Lists!$L$2:$L$10</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$M$1:$M$22</formula1>
+      <formula1>=Lists!$M$2:$M$23</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." promptTitle="Pick or type" prompt="Pick from the list, or type it." type="list">
-      <formula1>=Lists!$N$1:$N$2</formula1>
+      <formula1>=Lists!$N$2:$N$3</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$O$1:$O$13</formula1>
+      <formula1>=Lists!$O$2:$O$14</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$P$1:$P$3</formula1>
+      <formula1>=Lists!$P$2:$P$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18064,808 +18064,890 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Design firm</t>
+          <t>-</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>@roles</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>@cities</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>@cities</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Roshan Bisani</t>
+          <t>@team</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>@architect_ratings</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>@sources</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>@client_statuses</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>EGO direct</t>
+          <t>@relationships</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>@roles</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Individual</t>
+          <t>@client_types</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>@cities</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Roshan Bisani</t>
+          <t>@team</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>@sources</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>@client_statuses</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Design firm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Roshan Bisani</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>EGO direct</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Roshan Bisani</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Architect</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Navi Mumbai</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Navi Mumbai</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>ZippyScale Admin</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Google Ads</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Prospect</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Via dealer</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Homeowner</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Navi Mumbai</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>ZippyScale Admin</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Google Ads</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Prospect</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Director</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Thane</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Thane</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Inactive</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Director</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Builder</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Thane</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Inactive</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Thane</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Thane</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Inactive</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Contractor</t>
+          <t>Builder</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Thane</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Purchase</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nashik</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Nashik</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>IndiaMART</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Purchase</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Contractor</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Nashik</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>IndiaMART</t>
+          <t>WhatsApp</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>Accounts</t>
+          <t>Purchase</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nagpur</t>
+          <t>Nashik</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Nagpur</t>
+          <t>Nashik</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>JustDial</t>
+          <t>IndiaMART</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Accounts</t>
+          <t>Purchase</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Corporate</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Nagpur</t>
+          <t>Nashik</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>JustDial</t>
+          <t>IndiaMART</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Store manager</t>
+          <t>Accounts</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Ahmedabad</t>
+          <t>Nagpur</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ahmedabad</t>
+          <t>Nagpur</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>QR code</t>
+          <t>JustDial</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Store manager</t>
+          <t>Accounts</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Retail chain</t>
+          <t>Corporate</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Ahmedabad</t>
+          <t>Nagpur</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>QR code</t>
+          <t>JustDial</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Store manager</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Surat</t>
+          <t>Ahmedabad</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Surat</t>
+          <t>Ahmedabad</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Walk-in</t>
+          <t>QR code</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Store manager</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Institution</t>
+          <t>Retail chain</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Surat</t>
+          <t>Ahmedabad</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Walk-in</t>
+          <t>QR code</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>Telecaller</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Vadodara</t>
+          <t>Surat</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Vadodara</t>
+          <t>Surat</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Referral</t>
+          <t>Walk-in</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Telecaller</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Other firm</t>
+          <t>Institution</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Vadodara</t>
+          <t>Surat</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Referral</t>
+          <t>Walk-in</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Telecaller</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goa</t>
+          <t>Vadodara</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Goa</t>
+          <t>Vadodara</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Field visit</t>
+          <t>Referral</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Telecaller</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Other firm</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Goa</t>
+          <t>Vadodara</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Field visit</t>
+          <t>Referral</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>Site engineer</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Goa</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Goa</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Field visit</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Site engineer</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Goa</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Field visit</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>Project manager</t>
+          <t>Site engineer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Existing relationship</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Project manager</t>
+          <t>Site engineer</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Existing relationship</t>
+          <t>Architect</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>Senior architect</t>
+          <t>Project manager</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Existing relationship</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Senior architect</t>
+          <t>Project manager</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Existing relationship</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Senior architect</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Other</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Senior architect</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Other</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>New Delhi</t>
+          <t>Kochi</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>New Delhi</t>
+          <t>Kochi</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>New Delhi</t>
+          <t>Kochi</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
+          <t>Interior designer</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>New Delhi</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>New Delhi</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Interior designer</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>New Delhi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Gurugram</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Gurugram</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>Gurugram</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Noida</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Noida</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Noida</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="C18" t="inlineStr">
         <is>
-          <t>Jaipur</t>
+          <t>Noida</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Jaipur</t>
+          <t>Noida</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Jaipur</t>
+          <t>Noida</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="C19" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>Jaipur</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>Jaipur</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>Jaipur</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="C20" t="inlineStr">
         <is>
-          <t>Lucknow</t>
+          <t>Chandigarh</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Lucknow</t>
+          <t>Chandigarh</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Lucknow</t>
+          <t>Chandigarh</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="C21" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Lucknow</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Lucknow</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Lucknow</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="C22" t="inlineStr">
         <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="C23" t="inlineStr">
+        <is>
           <t>Indore</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Indore</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>Indore</t>
         </is>

</xml_diff>

<commit_message>
EGO live: onboarding answers (dealer service, EGO order flow, payments, schemes, charges, lost details)
</commit_message>
<xml_diff>
--- a/ego/Big-E-Upload-Template.xlsx
+++ b/ego/Big-E-Upload-Template.xlsx
@@ -6985,7 +6985,7 @@
       <formula1>=Lists!$F$2:$F$4</formula1>
     </dataValidation>
     <dataValidation sqref="R2:R1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$G$2:$G$14</formula1>
+      <formula1>=Lists!$G$2:$G$16</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$H$2:$H$4</formula1>
@@ -18048,7 +18048,7 @@
       <formula1>=Lists!$N$2:$N$3</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$O$2:$O$14</formula1>
+      <formula1>=Lists!$O$2:$O$16</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$P$2:$P$4</formula1>
@@ -18514,7 +18514,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>QR code</t>
+          <t>Runo</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -18534,7 +18534,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>QR code</t>
+          <t>Runo</t>
         </is>
       </c>
     </row>
@@ -18556,7 +18556,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Walk-in</t>
+          <t>Sales Diary</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -18576,7 +18576,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Walk-in</t>
+          <t>Sales Diary</t>
         </is>
       </c>
     </row>
@@ -18598,7 +18598,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Referral</t>
+          <t>QR code</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -18618,7 +18618,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Referral</t>
+          <t>QR code</t>
         </is>
       </c>
     </row>
@@ -18640,7 +18640,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Field visit</t>
+          <t>Walk-in</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -18655,7 +18655,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Field visit</t>
+          <t>Walk-in</t>
         </is>
       </c>
     </row>
@@ -18677,7 +18677,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Referral</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -18692,7 +18692,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Referral</t>
         </is>
       </c>
     </row>
@@ -18714,7 +18714,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Existing relationship</t>
+          <t>Field visit</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -18729,7 +18729,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Existing relationship</t>
+          <t>Field visit</t>
         </is>
       </c>
     </row>
@@ -18751,7 +18751,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -18766,7 +18766,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Architect</t>
         </is>
       </c>
     </row>
@@ -18786,6 +18786,11 @@
           <t>Kochi</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Existing relationship</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
           <t>Architect</t>
@@ -18794,6 +18799,11 @@
       <c r="M15" t="inlineStr">
         <is>
           <t>Kochi</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Existing relationship</t>
         </is>
       </c>
     </row>
@@ -18813,6 +18823,11 @@
           <t>New Delhi</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr">
         <is>
           <t>Interior designer</t>
@@ -18821,6 +18836,11 @@
       <c r="M16" t="inlineStr">
         <is>
           <t>New Delhi</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Other</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EGO live: Excel files with the team
</commit_message>
<xml_diff>
--- a/ego/Big-E-Upload-Template.xlsx
+++ b/ego/Big-E-Upload-Template.xlsx
@@ -6979,7 +6979,7 @@
       <formula1>=Lists!$D$2:$D$23</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." promptTitle="Pick or type" prompt="Pick from the list, or type it." type="list">
-      <formula1>=Lists!$E$2:$E$3</formula1>
+      <formula1>=Lists!$E$2:$E$28</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$F$2:$F$4</formula1>
@@ -18045,7 +18045,7 @@
       <formula1>=Lists!$M$2:$M$23</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." promptTitle="Pick or type" prompt="Pick from the list, or type it." type="list">
-      <formula1>=Lists!$N$2:$N$3</formula1>
+      <formula1>=Lists!$N$2:$N$28</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$O$2:$O$16</formula1>
@@ -18064,7 +18064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18172,7 +18172,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Roshan Bisani</t>
+          <t>Aliza Arif Mukri</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -18217,7 +18217,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Roshan Bisani</t>
+          <t>Aliza Arif Mukri</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -18254,7 +18254,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ZippyScale Admin</t>
+          <t>Anjali Maurya</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -18299,7 +18299,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>ZippyScale Admin</t>
+          <t>Anjali Maurya</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -18329,6 +18329,11 @@
           <t>Thane</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Basanti Damai</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>C</t>
@@ -18357,6 +18362,11 @@
       <c r="M4" t="inlineStr">
         <is>
           <t>Thane</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Basanti Damai</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -18386,6 +18396,11 @@
           <t>Pune</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Bharti Kapoor</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>WhatsApp</t>
@@ -18404,6 +18419,11 @@
       <c r="M5" t="inlineStr">
         <is>
           <t>Pune</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Bharti Kapoor</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -18428,6 +18448,11 @@
           <t>Nashik</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Dattatray Sudam Gadhave</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>IndiaMART</t>
@@ -18446,6 +18471,11 @@
       <c r="M6" t="inlineStr">
         <is>
           <t>Nashik</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Dattatray Sudam Gadhave</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -18470,6 +18500,11 @@
           <t>Nagpur</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Hardeep Kaur</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>JustDial</t>
@@ -18488,6 +18523,11 @@
       <c r="M7" t="inlineStr">
         <is>
           <t>Nagpur</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Hardeep Kaur</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -18512,6 +18552,11 @@
           <t>Ahmedabad</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Joycee Ashok Rokade</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>Runo</t>
@@ -18530,6 +18575,11 @@
       <c r="M8" t="inlineStr">
         <is>
           <t>Ahmedabad</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Joycee Ashok Rokade</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -18554,6 +18604,11 @@
           <t>Surat</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Jyoti Andrews</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>Sales Diary</t>
@@ -18572,6 +18627,11 @@
       <c r="M9" t="inlineStr">
         <is>
           <t>Surat</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Jyoti Andrews</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -18596,6 +18656,11 @@
           <t>Vadodara</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Kishor Mhaske</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>QR code</t>
@@ -18614,6 +18679,11 @@
       <c r="M10" t="inlineStr">
         <is>
           <t>Vadodara</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Kishor Mhaske</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -18638,6 +18708,11 @@
           <t>Goa</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Madan Kolkur</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>Walk-in</t>
@@ -18651,6 +18726,11 @@
       <c r="M11" t="inlineStr">
         <is>
           <t>Goa</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Madan Kolkur</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -18675,6 +18755,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Nilesh Khandkar</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
           <t>Referral</t>
@@ -18688,6 +18773,11 @@
       <c r="M12" t="inlineStr">
         <is>
           <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Nilesh Khandkar</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -18712,6 +18802,11 @@
           <t>Chennai</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Palash Sharma</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>Field visit</t>
@@ -18725,6 +18820,11 @@
       <c r="M13" t="inlineStr">
         <is>
           <t>Chennai</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Palash Sharma</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -18749,6 +18849,11 @@
           <t>Hyderabad</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Pankaj Kumar</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>Architect</t>
@@ -18762,6 +18867,11 @@
       <c r="M14" t="inlineStr">
         <is>
           <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Pankaj Kumar</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -18786,6 +18896,11 @@
           <t>Kochi</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Paramjeet Saini</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>Existing relationship</t>
@@ -18799,6 +18914,11 @@
       <c r="M15" t="inlineStr">
         <is>
           <t>Kochi</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Paramjeet Saini</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -18823,6 +18943,11 @@
           <t>New Delhi</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Pradeep Yashwantrao Washimkar</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>Other</t>
@@ -18836,6 +18961,11 @@
       <c r="M16" t="inlineStr">
         <is>
           <t>New Delhi</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Pradeep Yashwantrao Washimkar</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -18860,6 +18990,11 @@
           <t>Gurugram</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Pradnya Kaustubh Khare</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
           <t>Other</t>
@@ -18868,6 +19003,11 @@
       <c r="M17" t="inlineStr">
         <is>
           <t>Gurugram</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Pradnya Kaustubh Khare</t>
         </is>
       </c>
     </row>
@@ -18882,9 +19022,19 @@
           <t>Noida</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Pravez Khan</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr">
         <is>
           <t>Noida</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Pravez Khan</t>
         </is>
       </c>
     </row>
@@ -18899,9 +19049,19 @@
           <t>Jaipur</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Pravin Shingare</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr">
         <is>
           <t>Jaipur</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Pravin Shingare</t>
         </is>
       </c>
     </row>
@@ -18916,9 +19076,19 @@
           <t>Chandigarh</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Rahul Bajpai</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr">
         <is>
           <t>Chandigarh</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Rahul Bajpai</t>
         </is>
       </c>
     </row>
@@ -18933,9 +19103,19 @@
           <t>Lucknow</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Roshan Bisani</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>Lucknow</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Roshan Bisani</t>
         </is>
       </c>
     </row>
@@ -18950,9 +19130,19 @@
           <t>Kolkata</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Salimullah</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr">
         <is>
           <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Salimullah</t>
         </is>
       </c>
     </row>
@@ -18967,9 +19157,79 @@
           <t>Indore</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Sanket Jage</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>Indore</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Sanket Jage</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sunil Dongrani</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Sunil Dongrani</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Tarun Goverkar</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Tarun Goverkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Vijay Pandhre</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Vijay Pandhre</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Virendra Pratap Ram Singh</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Virendra Pratap Ram Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ZippyScale Admin</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>ZippyScale Admin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EGO Master R2b: + Requirement, My requirements, My numbers, weak network queue, offline open; build d75ca60636
</commit_message>
<xml_diff>
--- a/ego/Big-E-Upload-Template.xlsx
+++ b/ego/Big-E-Upload-Template.xlsx
@@ -7053,7 +7053,7 @@
       <formula1>=Lists!$G$2:$G$4</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$H$2:$H$16</formula1>
+      <formula1>=Lists!$H$2:$H$17</formula1>
     </dataValidation>
     <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$I$2:$I$4</formula1>
@@ -18184,7 +18184,7 @@
       <formula1>=Lists!$P$2:$P$28</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$Q$2:$Q$16</formula1>
+      <formula1>=Lists!$Q$2:$Q$17</formula1>
     </dataValidation>
     <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$R$2:$R$4</formula1>
@@ -19127,7 +19127,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Field sales</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -19152,7 +19152,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Field sales</t>
         </is>
       </c>
     </row>
@@ -19184,7 +19184,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Existing relationship</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -19209,7 +19209,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Existing relationship</t>
+          <t>Architect</t>
         </is>
       </c>
     </row>
@@ -19241,7 +19241,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Existing relationship</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -19266,7 +19266,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Existing relationship</t>
         </is>
       </c>
     </row>
@@ -19296,6 +19296,11 @@
           <t>Pradnya Kaustubh Khare</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>Other</t>
@@ -19314,6 +19319,11 @@
       <c r="P17" t="inlineStr">
         <is>
           <t>Pradnya Kaustubh Khare</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Other</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EGO Master e36df50dbc (25 Oct): role changes management only, no deletes, India cities, target original kept, admin resets limited, crash reports name the line
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ego/Big-E-Upload-Template.xlsx
+++ b/ego/Big-E-Upload-Template.xlsx
@@ -7224,13 +7224,13 @@
       <formula1>=Lists!$B$2:$B$17</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$C$2:$C$23</formula1>
+      <formula1>=Lists!$C$2:$C$161</formula1>
     </dataValidation>
     <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$D$2:$D$37</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." promptTitle="Pick or type" prompt="Pick from the list, or type several separated by commas." type="list">
-      <formula1>=Lists!$E$2:$E$23</formula1>
+      <formula1>=Lists!$E$2:$E$161</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." promptTitle="Pick or type" prompt="Pick from the list, or type it." type="list">
       <formula1>=Lists!$F$2:$F$28</formula1>
@@ -18976,13 +18976,13 @@
       <formula1>=Lists!$N$2:$N$17</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$O$2:$O$23</formula1>
+      <formula1>=Lists!$O$2:$O$161</formula1>
     </dataValidation>
     <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$P$2:$P$37</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." promptTitle="Pick or type" prompt="Pick from the list, or type several separated by commas." type="list">
-      <formula1>=Lists!$Q$2:$Q$23</formula1>
+      <formula1>=Lists!$Q$2:$Q$161</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." promptTitle="Pick or type" prompt="Pick from the list, or type it." type="list">
       <formula1>=Lists!$R$2:$R$28</formula1>
@@ -30113,7 +30113,7 @@
       <formula1>=Lists!$Y$2:$Y$10</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$Z$2:$Z$23</formula1>
+      <formula1>=Lists!$Z$2:$Z$161</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$AA$2:$AA$37</formula1>
@@ -30138,7 +30138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD37"/>
+  <dimension ref="A1:AD161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32298,26 +32298,51 @@
       </c>
     </row>
     <row r="24">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Kalyan</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>Meghalaya</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Kalyan</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>Sunil Dongrani</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Kalyan</t>
+        </is>
+      </c>
       <c r="P24" t="inlineStr">
         <is>
           <t>Meghalaya</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Kalyan</t>
+        </is>
+      </c>
       <c r="R24" t="inlineStr">
         <is>
           <t>Sunil Dongrani</t>
         </is>
       </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>Kalyan</t>
+        </is>
+      </c>
       <c r="AA24" t="inlineStr">
         <is>
           <t>Meghalaya</t>
@@ -32330,26 +32355,51 @@
       </c>
     </row>
     <row r="25">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Dombivli</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>Mizoram</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Dombivli</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>Tarun Goverkar</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Dombivli</t>
+        </is>
+      </c>
       <c r="P25" t="inlineStr">
         <is>
           <t>Mizoram</t>
         </is>
       </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Dombivli</t>
+        </is>
+      </c>
       <c r="R25" t="inlineStr">
         <is>
           <t>Tarun Goverkar</t>
         </is>
       </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>Dombivli</t>
+        </is>
+      </c>
       <c r="AA25" t="inlineStr">
         <is>
           <t>Mizoram</t>
@@ -32362,26 +32412,51 @@
       </c>
     </row>
     <row r="26">
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>Nagaland</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Vijay Pandhre</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
       <c r="P26" t="inlineStr">
         <is>
           <t>Nagaland</t>
         </is>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
       <c r="R26" t="inlineStr">
         <is>
           <t>Vijay Pandhre</t>
         </is>
       </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
       <c r="AA26" t="inlineStr">
         <is>
           <t>Nagaland</t>
@@ -32394,26 +32469,51 @@
       </c>
     </row>
     <row r="27">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Vasai-Virar</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>Odisha</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Vasai-Virar</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Virendra Pratap Ram Singh</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Vasai-Virar</t>
+        </is>
+      </c>
       <c r="P27" t="inlineStr">
         <is>
           <t>Odisha</t>
         </is>
       </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Vasai-Virar</t>
+        </is>
+      </c>
       <c r="R27" t="inlineStr">
         <is>
           <t>Virendra Pratap Ram Singh</t>
         </is>
       </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>Vasai-Virar</t>
+        </is>
+      </c>
       <c r="AA27" t="inlineStr">
         <is>
           <t>Odisha</t>
@@ -32426,26 +32526,51 @@
       </c>
     </row>
     <row r="28">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Panvel</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>Puducherry</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Panvel</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>ZippyScale Admin</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Panvel</t>
+        </is>
+      </c>
       <c r="P28" t="inlineStr">
         <is>
           <t>Puducherry</t>
         </is>
       </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Panvel</t>
+        </is>
+      </c>
       <c r="R28" t="inlineStr">
         <is>
           <t>ZippyScale Admin</t>
         </is>
       </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>Panvel</t>
+        </is>
+      </c>
       <c r="AA28" t="inlineStr">
         <is>
           <t>Puducherry</t>
@@ -32458,16 +32583,41 @@
       </c>
     </row>
     <row r="29">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Mira-Bhayandar</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>Punjab</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Mira-Bhayandar</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Mira-Bhayandar</t>
+        </is>
+      </c>
       <c r="P29" t="inlineStr">
         <is>
           <t>Punjab</t>
         </is>
       </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Mira-Bhayandar</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>Mira-Bhayandar</t>
+        </is>
+      </c>
       <c r="AA29" t="inlineStr">
         <is>
           <t>Punjab</t>
@@ -32475,16 +32625,41 @@
       </c>
     </row>
     <row r="30">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Ulhasnagar</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>Rajasthan</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Ulhasnagar</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Ulhasnagar</t>
+        </is>
+      </c>
       <c r="P30" t="inlineStr">
         <is>
           <t>Rajasthan</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Ulhasnagar</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>Ulhasnagar</t>
+        </is>
+      </c>
       <c r="AA30" t="inlineStr">
         <is>
           <t>Rajasthan</t>
@@ -32492,16 +32667,41 @@
       </c>
     </row>
     <row r="31">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Pimpri-Chinchwad</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>Sikkim</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Pimpri-Chinchwad</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Pimpri-Chinchwad</t>
+        </is>
+      </c>
       <c r="P31" t="inlineStr">
         <is>
           <t>Sikkim</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Pimpri-Chinchwad</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>Pimpri-Chinchwad</t>
+        </is>
+      </c>
       <c r="AA31" t="inlineStr">
         <is>
           <t>Sikkim</t>
@@ -32509,16 +32709,41 @@
       </c>
     </row>
     <row r="32">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Aurangabad</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>Tamil Nadu</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Aurangabad</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Aurangabad</t>
+        </is>
+      </c>
       <c r="P32" t="inlineStr">
         <is>
           <t>Tamil Nadu</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Aurangabad</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>Aurangabad</t>
+        </is>
+      </c>
       <c r="AA32" t="inlineStr">
         <is>
           <t>Tamil Nadu</t>
@@ -32526,16 +32751,41 @@
       </c>
     </row>
     <row r="33">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Solapur</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>Telangana</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Solapur</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Solapur</t>
+        </is>
+      </c>
       <c r="P33" t="inlineStr">
         <is>
           <t>Telangana</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Solapur</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>Solapur</t>
+        </is>
+      </c>
       <c r="AA33" t="inlineStr">
         <is>
           <t>Telangana</t>
@@ -32543,16 +32793,41 @@
       </c>
     </row>
     <row r="34">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Kolhapur</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>Tripura</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Kolhapur</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Kolhapur</t>
+        </is>
+      </c>
       <c r="P34" t="inlineStr">
         <is>
           <t>Tripura</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Kolhapur</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>Kolhapur</t>
+        </is>
+      </c>
       <c r="AA34" t="inlineStr">
         <is>
           <t>Tripura</t>
@@ -32560,16 +32835,41 @@
       </c>
     </row>
     <row r="35">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Sangli</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>Uttar Pradesh</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Sangli</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Sangli</t>
+        </is>
+      </c>
       <c r="P35" t="inlineStr">
         <is>
           <t>Uttar Pradesh</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Sangli</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>Sangli</t>
+        </is>
+      </c>
       <c r="AA35" t="inlineStr">
         <is>
           <t>Uttar Pradesh</t>
@@ -32577,16 +32877,41 @@
       </c>
     </row>
     <row r="36">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Amravati</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>Uttarakhand</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Amravati</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Amravati</t>
+        </is>
+      </c>
       <c r="P36" t="inlineStr">
         <is>
           <t>Uttarakhand</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Amravati</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>Amravati</t>
+        </is>
+      </c>
       <c r="AA36" t="inlineStr">
         <is>
           <t>Uttarakhand</t>
@@ -32594,19 +32919,3392 @@
       </c>
     </row>
     <row r="37">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Akola</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>West Bengal</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Akola</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Akola</t>
+        </is>
+      </c>
       <c r="P37" t="inlineStr">
         <is>
           <t>West Bengal</t>
         </is>
       </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Akola</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>Akola</t>
+        </is>
+      </c>
       <c r="AA37" t="inlineStr">
         <is>
           <t>West Bengal</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Jalgaon</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Jalgaon</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Jalgaon</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Jalgaon</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>Jalgaon</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Ahmednagar</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Ahmednagar</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Ahmednagar</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Ahmednagar</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>Ahmednagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Latur</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Latur</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Latur</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Latur</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Latur</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nanded</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Nanded</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Nanded</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Nanded</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Nanded</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Satara</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Satara</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Satara</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Satara</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>Satara</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Ratnagiri</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Ratnagiri</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Ratnagiri</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Ratnagiri</t>
+        </is>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>Ratnagiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Rajkot</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Rajkot</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Rajkot</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Rajkot</t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>Rajkot</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Gandhinagar</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Gandhinagar</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Gandhinagar</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Gandhinagar</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>Gandhinagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Bhavnagar</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Bhavnagar</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Bhavnagar</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Bhavnagar</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>Bhavnagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Jamnagar</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Jamnagar</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Jamnagar</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Jamnagar</t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>Jamnagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Anand</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Anand</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Anand</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Anand</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>Anand</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Vapi</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Vapi</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Vapi</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Vapi</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>Vapi</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Bharuch</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Bharuch</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Bharuch</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Bharuch</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>Bharuch</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Mehsana</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Mehsana</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Mehsana</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Mehsana</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>Mehsana</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Junagadh</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Junagadh</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Junagadh</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Junagadh</t>
+        </is>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>Junagadh</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Gandhidham</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Gandhidham</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Gandhidham</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Gandhidham</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>Gandhidham</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Panaji</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Panaji</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Panaji</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Panaji</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>Panaji</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Margao</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Margao</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Margao</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Margao</t>
+        </is>
+      </c>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>Margao</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="Z56" t="inlineStr">
+        <is>
+          <t>Vasco da Gama</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Mapusa</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Mapusa</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Mapusa</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Mapusa</t>
+        </is>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>Mapusa</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Silvassa</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Silvassa</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>Silvassa</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Silvassa</t>
+        </is>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>Silvassa</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Daman</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Daman</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>Daman</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Daman</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>Daman</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Mysuru</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Mysuru</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Mysuru</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Mysuru</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>Mysuru</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Mangaluru</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Mangaluru</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>Mangaluru</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Mangaluru</t>
+        </is>
+      </c>
+      <c r="Z61" t="inlineStr">
+        <is>
+          <t>Mangaluru</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Hubballi</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Hubballi</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>Hubballi</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Hubballi</t>
+        </is>
+      </c>
+      <c r="Z62" t="inlineStr">
+        <is>
+          <t>Hubballi</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Belagavi</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Belagavi</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Belagavi</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Belagavi</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>Belagavi</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Davanagere</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Davanagere</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>Davanagere</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Davanagere</t>
+        </is>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>Davanagere</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Kalaburagi</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Kalaburagi</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>Kalaburagi</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Kalaburagi</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>Kalaburagi</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Udupi</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Udupi</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>Udupi</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Udupi</t>
+        </is>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>Udupi</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Madurai</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Madurai</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>Madurai</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Madurai</t>
+        </is>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>Madurai</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Tiruchirappalli</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Tiruchirappalli</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>Tiruchirappalli</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>Tiruchirappalli</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>Tiruchirappalli</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Salem</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Salem</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>Salem</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Salem</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>Salem</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Tiruppur</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Tiruppur</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Tiruppur</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Tiruppur</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>Tiruppur</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Vellore</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Vellore</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Vellore</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Vellore</t>
+        </is>
+      </c>
+      <c r="Z73" t="inlineStr">
+        <is>
+          <t>Vellore</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Tirunelveli</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Tirunelveli</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>Tirunelveli</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>Tirunelveli</t>
+        </is>
+      </c>
+      <c r="Z74" t="inlineStr">
+        <is>
+          <t>Tirunelveli</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Hosur</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Hosur</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>Hosur</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>Hosur</t>
+        </is>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>Hosur</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Secunderabad</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Secunderabad</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>Secunderabad</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>Secunderabad</t>
+        </is>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>Secunderabad</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>Khammam</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>Visakhapatnam</t>
+        </is>
+      </c>
+      <c r="Z81" t="inlineStr">
+        <is>
+          <t>Visakhapatnam</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Guntur</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Guntur</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>Guntur</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>Guntur</t>
+        </is>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
+          <t>Guntur</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Nellore</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Nellore</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>Nellore</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>Nellore</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>Nellore</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Tirupati</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Tirupati</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>Tirupati</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>Tirupati</t>
+        </is>
+      </c>
+      <c r="Z85" t="inlineStr">
+        <is>
+          <t>Tirupati</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Kakinada</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Kakinada</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>Kakinada</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>Kakinada</t>
+        </is>
+      </c>
+      <c r="Z86" t="inlineStr">
+        <is>
+          <t>Kakinada</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Rajahmundry</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Rajahmundry</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>Rajahmundry</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>Rajahmundry</t>
+        </is>
+      </c>
+      <c r="Z87" t="inlineStr">
+        <is>
+          <t>Rajahmundry</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Kurnool</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Kurnool</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>Kurnool</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>Kurnool</t>
+        </is>
+      </c>
+      <c r="Z88" t="inlineStr">
+        <is>
+          <t>Kurnool</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+      <c r="Z89" t="inlineStr">
+        <is>
+          <t>Anantapur</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Thiruvananthapuram</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Thiruvananthapuram</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>Thiruvananthapuram</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>Thiruvananthapuram</t>
+        </is>
+      </c>
+      <c r="Z90" t="inlineStr">
+        <is>
+          <t>Thiruvananthapuram</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Kozhikode</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Kozhikode</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>Kozhikode</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>Kozhikode</t>
+        </is>
+      </c>
+      <c r="Z91" t="inlineStr">
+        <is>
+          <t>Kozhikode</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Thrissur</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Thrissur</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>Thrissur</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>Thrissur</t>
+        </is>
+      </c>
+      <c r="Z92" t="inlineStr">
+        <is>
+          <t>Thrissur</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Kollam</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Kollam</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>Kollam</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>Kollam</t>
+        </is>
+      </c>
+      <c r="Z93" t="inlineStr">
+        <is>
+          <t>Kollam</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Kannur</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Kannur</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>Kannur</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>Kannur</t>
+        </is>
+      </c>
+      <c r="Z94" t="inlineStr">
+        <is>
+          <t>Kannur</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Puducherry</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Puducherry</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>Puducherry</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>Puducherry</t>
+        </is>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>Puducherry</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Faridabad</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Faridabad</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>Faridabad</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>Faridabad</t>
+        </is>
+      </c>
+      <c r="Z97" t="inlineStr">
+        <is>
+          <t>Faridabad</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Panipat</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Panipat</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>Panipat</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>Panipat</t>
+        </is>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>Panipat</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Sonipat</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Sonipat</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>Sonipat</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>Sonipat</t>
+        </is>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>Sonipat</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Ambala</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Ambala</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>Ambala</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>Ambala</t>
+        </is>
+      </c>
+      <c r="Z100" t="inlineStr">
+        <is>
+          <t>Ambala</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Karnal</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Karnal</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>Karnal</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>Karnal</t>
+        </is>
+      </c>
+      <c r="Z101" t="inlineStr">
+        <is>
+          <t>Karnal</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Hisar</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Hisar</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>Hisar</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>Hisar</t>
+        </is>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>Hisar</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Rohtak</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Rohtak</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>Rohtak</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>Rohtak</t>
+        </is>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>Rohtak</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Ghaziabad</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Ghaziabad</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>Ghaziabad</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>Ghaziabad</t>
+        </is>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>Ghaziabad</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Greater Noida</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Greater Noida</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>Greater Noida</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>Greater Noida</t>
+        </is>
+      </c>
+      <c r="Z105" t="inlineStr">
+        <is>
+          <t>Greater Noida</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Kanpur</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Kanpur</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>Kanpur</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>Kanpur</t>
+        </is>
+      </c>
+      <c r="Z106" t="inlineStr">
+        <is>
+          <t>Kanpur</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Agra</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Agra</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>Agra</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>Agra</t>
+        </is>
+      </c>
+      <c r="Z107" t="inlineStr">
+        <is>
+          <t>Agra</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Varanasi</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Varanasi</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>Varanasi</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>Varanasi</t>
+        </is>
+      </c>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t>Varanasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Meerut</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Meerut</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>Meerut</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>Meerut</t>
+        </is>
+      </c>
+      <c r="Z109" t="inlineStr">
+        <is>
+          <t>Meerut</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Prayagraj</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Prayagraj</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>Prayagraj</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>Prayagraj</t>
+        </is>
+      </c>
+      <c r="Z110" t="inlineStr">
+        <is>
+          <t>Prayagraj</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Bareilly</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Bareilly</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>Bareilly</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>Bareilly</t>
+        </is>
+      </c>
+      <c r="Z111" t="inlineStr">
+        <is>
+          <t>Bareilly</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Aligarh</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Aligarh</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>Aligarh</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>Aligarh</t>
+        </is>
+      </c>
+      <c r="Z112" t="inlineStr">
+        <is>
+          <t>Aligarh</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Moradabad</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Moradabad</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>Moradabad</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>Moradabad</t>
+        </is>
+      </c>
+      <c r="Z113" t="inlineStr">
+        <is>
+          <t>Moradabad</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Gorakhpur</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Gorakhpur</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Gorakhpur</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>Gorakhpur</t>
+        </is>
+      </c>
+      <c r="Z114" t="inlineStr">
+        <is>
+          <t>Gorakhpur</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Jodhpur</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Jodhpur</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>Jodhpur</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>Jodhpur</t>
+        </is>
+      </c>
+      <c r="Z115" t="inlineStr">
+        <is>
+          <t>Jodhpur</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Udaipur</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Udaipur</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>Udaipur</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>Udaipur</t>
+        </is>
+      </c>
+      <c r="Z116" t="inlineStr">
+        <is>
+          <t>Udaipur</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Kota</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Kota</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>Kota</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>Kota</t>
+        </is>
+      </c>
+      <c r="Z117" t="inlineStr">
+        <is>
+          <t>Kota</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Ajmer</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Ajmer</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>Ajmer</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>Ajmer</t>
+        </is>
+      </c>
+      <c r="Z118" t="inlineStr">
+        <is>
+          <t>Ajmer</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Bikaner</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Bikaner</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>Bikaner</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>Bikaner</t>
+        </is>
+      </c>
+      <c r="Z119" t="inlineStr">
+        <is>
+          <t>Bikaner</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Ludhiana</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Ludhiana</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>Ludhiana</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>Ludhiana</t>
+        </is>
+      </c>
+      <c r="Z120" t="inlineStr">
+        <is>
+          <t>Ludhiana</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Amritsar</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Amritsar</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>Amritsar</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>Amritsar</t>
+        </is>
+      </c>
+      <c r="Z121" t="inlineStr">
+        <is>
+          <t>Amritsar</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Jalandhar</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Jalandhar</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>Jalandhar</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>Jalandhar</t>
+        </is>
+      </c>
+      <c r="Z122" t="inlineStr">
+        <is>
+          <t>Jalandhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Mohali</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Mohali</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>Mohali</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>Mohali</t>
+        </is>
+      </c>
+      <c r="Z123" t="inlineStr">
+        <is>
+          <t>Mohali</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Patiala</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Patiala</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>Patiala</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>Patiala</t>
+        </is>
+      </c>
+      <c r="Z124" t="inlineStr">
+        <is>
+          <t>Patiala</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Bathinda</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Bathinda</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>Bathinda</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>Bathinda</t>
+        </is>
+      </c>
+      <c r="Z125" t="inlineStr">
+        <is>
+          <t>Bathinda</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Dehradun</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Dehradun</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>Dehradun</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>Dehradun</t>
+        </is>
+      </c>
+      <c r="Z126" t="inlineStr">
+        <is>
+          <t>Dehradun</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Haridwar</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Haridwar</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>Haridwar</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>Haridwar</t>
+        </is>
+      </c>
+      <c r="Z127" t="inlineStr">
+        <is>
+          <t>Haridwar</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Haldwani</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Haldwani</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>Haldwani</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>Haldwani</t>
+        </is>
+      </c>
+      <c r="Z128" t="inlineStr">
+        <is>
+          <t>Haldwani</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Shimla</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Shimla</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>Shimla</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>Shimla</t>
+        </is>
+      </c>
+      <c r="Z129" t="inlineStr">
+        <is>
+          <t>Shimla</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Jammu</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Jammu</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>Jammu</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>Jammu</t>
+        </is>
+      </c>
+      <c r="Z130" t="inlineStr">
+        <is>
+          <t>Jammu</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Srinagar</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Srinagar</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>Srinagar</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>Srinagar</t>
+        </is>
+      </c>
+      <c r="Z131" t="inlineStr">
+        <is>
+          <t>Srinagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Howrah</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Howrah</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>Howrah</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>Howrah</t>
+        </is>
+      </c>
+      <c r="Z132" t="inlineStr">
+        <is>
+          <t>Howrah</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Durgapur</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Durgapur</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>Durgapur</t>
+        </is>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>Durgapur</t>
+        </is>
+      </c>
+      <c r="Z133" t="inlineStr">
+        <is>
+          <t>Durgapur</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Asansol</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Asansol</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>Asansol</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>Asansol</t>
+        </is>
+      </c>
+      <c r="Z134" t="inlineStr">
+        <is>
+          <t>Asansol</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Siliguri</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Siliguri</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>Siliguri</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>Siliguri</t>
+        </is>
+      </c>
+      <c r="Z135" t="inlineStr">
+        <is>
+          <t>Siliguri</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Bhubaneswar</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Bhubaneswar</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>Bhubaneswar</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>Bhubaneswar</t>
+        </is>
+      </c>
+      <c r="Z136" t="inlineStr">
+        <is>
+          <t>Bhubaneswar</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Cuttack</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Cuttack</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>Cuttack</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>Cuttack</t>
+        </is>
+      </c>
+      <c r="Z137" t="inlineStr">
+        <is>
+          <t>Cuttack</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Rourkela</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Rourkela</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>Rourkela</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>Rourkela</t>
+        </is>
+      </c>
+      <c r="Z138" t="inlineStr">
+        <is>
+          <t>Rourkela</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Patna</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Patna</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>Patna</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>Patna</t>
+        </is>
+      </c>
+      <c r="Z139" t="inlineStr">
+        <is>
+          <t>Patna</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Gaya</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Gaya</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>Gaya</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>Gaya</t>
+        </is>
+      </c>
+      <c r="Z140" t="inlineStr">
+        <is>
+          <t>Gaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Muzaffarpur</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Muzaffarpur</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>Muzaffarpur</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>Muzaffarpur</t>
+        </is>
+      </c>
+      <c r="Z141" t="inlineStr">
+        <is>
+          <t>Muzaffarpur</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Ranchi</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Ranchi</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>Ranchi</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>Ranchi</t>
+        </is>
+      </c>
+      <c r="Z142" t="inlineStr">
+        <is>
+          <t>Ranchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Jamshedpur</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Jamshedpur</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>Jamshedpur</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>Jamshedpur</t>
+        </is>
+      </c>
+      <c r="Z143" t="inlineStr">
+        <is>
+          <t>Jamshedpur</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Dhanbad</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Dhanbad</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>Dhanbad</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>Dhanbad</t>
+        </is>
+      </c>
+      <c r="Z144" t="inlineStr">
+        <is>
+          <t>Dhanbad</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Bokaro</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Bokaro</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>Bokaro</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>Bokaro</t>
+        </is>
+      </c>
+      <c r="Z145" t="inlineStr">
+        <is>
+          <t>Bokaro</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Guwahati</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Guwahati</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>Guwahati</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>Guwahati</t>
+        </is>
+      </c>
+      <c r="Z146" t="inlineStr">
+        <is>
+          <t>Guwahati</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Dibrugarh</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Dibrugarh</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>Dibrugarh</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>Dibrugarh</t>
+        </is>
+      </c>
+      <c r="Z147" t="inlineStr">
+        <is>
+          <t>Dibrugarh</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Silchar</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Silchar</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>Silchar</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>Silchar</t>
+        </is>
+      </c>
+      <c r="Z148" t="inlineStr">
+        <is>
+          <t>Silchar</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Shillong</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Shillong</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>Shillong</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>Shillong</t>
+        </is>
+      </c>
+      <c r="Z149" t="inlineStr">
+        <is>
+          <t>Shillong</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Agartala</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Agartala</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>Agartala</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>Agartala</t>
+        </is>
+      </c>
+      <c r="Z150" t="inlineStr">
+        <is>
+          <t>Agartala</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Imphal</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Imphal</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>Imphal</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>Imphal</t>
+        </is>
+      </c>
+      <c r="Z151" t="inlineStr">
+        <is>
+          <t>Imphal</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Gangtok</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Gangtok</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>Gangtok</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>Gangtok</t>
+        </is>
+      </c>
+      <c r="Z152" t="inlineStr">
+        <is>
+          <t>Gangtok</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Bhopal</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Bhopal</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>Bhopal</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>Bhopal</t>
+        </is>
+      </c>
+      <c r="Z153" t="inlineStr">
+        <is>
+          <t>Bhopal</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Jabalpur</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Jabalpur</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>Jabalpur</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>Jabalpur</t>
+        </is>
+      </c>
+      <c r="Z154" t="inlineStr">
+        <is>
+          <t>Jabalpur</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Gwalior</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Gwalior</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>Gwalior</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>Gwalior</t>
+        </is>
+      </c>
+      <c r="Z155" t="inlineStr">
+        <is>
+          <t>Gwalior</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Ujjain</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Ujjain</t>
+        </is>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>Ujjain</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>Ujjain</t>
+        </is>
+      </c>
+      <c r="Z156" t="inlineStr">
+        <is>
+          <t>Ujjain</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Sagar</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Sagar</t>
+        </is>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>Sagar</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>Sagar</t>
+        </is>
+      </c>
+      <c r="Z157" t="inlineStr">
+        <is>
+          <t>Sagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="Z158" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Bhilai</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Bhilai</t>
+        </is>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>Bhilai</t>
+        </is>
+      </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>Bhilai</t>
+        </is>
+      </c>
+      <c r="Z159" t="inlineStr">
+        <is>
+          <t>Bhilai</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Bilaspur</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Bilaspur</t>
+        </is>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>Bilaspur</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>Bilaspur</t>
+        </is>
+      </c>
+      <c r="Z160" t="inlineStr">
+        <is>
+          <t>Bilaspur</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Durg</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Durg</t>
+        </is>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>Durg</t>
+        </is>
+      </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>Durg</t>
+        </is>
+      </c>
+      <c r="Z161" t="inlineStr">
+        <is>
+          <t>Durg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EGO Master live build 0384f3e4c0: Sales model batch 1 (Leads), from growth-engine 5f4210a
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ego/Big-E-Upload-Template.xlsx
+++ b/ego/Big-E-Upload-Template.xlsx
@@ -7242,7 +7242,7 @@
       <formula1>='Dealer companies'!$B$3:$B$1000</formula1>
     </dataValidation>
     <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$H$2:$H$17</formula1>
+      <formula1>=Lists!$H$2:$H$18</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$I$2:$I$4</formula1>
@@ -18991,7 +18991,7 @@
       <formula1>=Lists!$S$2:$S$4</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$T$2:$T$17</formula1>
+      <formula1>=Lists!$T$2:$T$18</formula1>
     </dataValidation>
     <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$U$2:$U$4</formula1>
@@ -30122,7 +30122,7 @@
       <formula1>=Lists!$AB$2:$AB$28</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$AC$2:$AC$17</formula1>
+      <formula1>=Lists!$AC$2:$AC$18</formula1>
     </dataValidation>
     <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
       <formula1>=Lists!$AD$2:$AD$4</formula1>
@@ -31976,6 +31976,11 @@
           <t>Pravez Khan</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Exhibition</t>
+        </is>
+      </c>
       <c r="O18" t="inlineStr">
         <is>
           <t>Noida</t>
@@ -31996,6 +32001,11 @@
           <t>Pravez Khan</t>
         </is>
       </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Exhibition</t>
+        </is>
+      </c>
       <c r="Z18" t="inlineStr">
         <is>
           <t>Noida</t>
@@ -32009,6 +32019,11 @@
       <c r="AB18" t="inlineStr">
         <is>
           <t>Pravez Khan</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>Exhibition</t>
         </is>
       </c>
     </row>

</xml_diff>